<commit_message>
downloads: integrate 38 newly staged PDFs into fulltext corpus; update priority tracker to 241/300 (80.3%)
</commit_message>
<xml_diff>
--- a/08_docs/PROJECT_MASTER_TRACKER.xlsx
+++ b/08_docs/PROJECT_MASTER_TRACKER.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Repository of downloaded full-text PDFs (241 total, 202 priority)</t>
+          <t>Repository of downloaded full-text PDFs (280 total, 241 priority)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -671,12 +671,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Contains 241 validated PDFs named canonically by REC ID.</t>
+          <t>Contains 280 validated PDFs named canonically by REC ID.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Retrieve remaining 98 priority PDFs.</t>
+          <t>Retrieve remaining 59 priority PDFs.</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>UPDATED (Y=202, N=98)</t>
+          <t>UPDATED (Y=241, N=59)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Download remaining 98 PDFs.</t>
+          <t>Download remaining 59 priority PDFs.</t>
         </is>
       </c>
     </row>
@@ -4930,12 +4930,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1014.pdf</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10050355)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1014.pdf</t>
         </is>
       </c>
     </row>
@@ -6298,12 +6298,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1116.pdf</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10030205)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1116.pdf</t>
         </is>
       </c>
     </row>
@@ -6754,12 +6754,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1150.pdf</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10020097)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1150.pdf</t>
         </is>
       </c>
     </row>
@@ -6982,12 +6982,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1167.pdf</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/electronics15061207)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1167.pdf</t>
         </is>
       </c>
     </row>
@@ -7039,12 +7039,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1171.pdf</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10080611)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1171.pdf</t>
         </is>
       </c>
     </row>
@@ -7210,12 +7210,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1208.pdf</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10040273)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1208.pdf</t>
         </is>
       </c>
     </row>
@@ -7324,12 +7324,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1223.pdf</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10070535)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1223.pdf</t>
         </is>
       </c>
     </row>
@@ -7552,12 +7552,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1252.pdf</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s26082436)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1252.pdf</t>
         </is>
       </c>
     </row>
@@ -7609,12 +7609,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1253.pdf</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -7639,7 +7639,7 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10060399)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1253.pdf</t>
         </is>
       </c>
     </row>
@@ -7666,12 +7666,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1274.pdf</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/rs18081133)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1274.pdf</t>
         </is>
       </c>
     </row>
@@ -7723,12 +7723,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1277.pdf</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10040252)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1277.pdf</t>
         </is>
       </c>
     </row>
@@ -7894,12 +7894,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1302.pdf</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/electronics15143064)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1302.pdf</t>
         </is>
       </c>
     </row>
@@ -7951,12 +7951,12 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1304.pdf</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -7981,7 +7981,7 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s26061984)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1304.pdf</t>
         </is>
       </c>
     </row>
@@ -8008,12 +8008,12 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1309.pdf</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10010065)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1309.pdf</t>
         </is>
       </c>
     </row>
@@ -8179,12 +8179,12 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1393.pdf</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -8209,7 +8209,7 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10010069)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1393.pdf</t>
         </is>
       </c>
     </row>
@@ -8521,12 +8521,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1453.pdf</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -8551,7 +8551,7 @@
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.1016/j.measurement.2026.121787)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1453.pdf</t>
         </is>
       </c>
     </row>
@@ -8578,12 +8578,12 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1454.pdf</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/electronics15101974)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1454.pdf</t>
         </is>
       </c>
     </row>
@@ -8692,12 +8692,12 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1512.pdf</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones10080561)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1512.pdf</t>
         </is>
       </c>
     </row>
@@ -9262,12 +9262,12 @@
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_0347.pdf</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from IEEE_Xplore (DOI: 10.1109/JSEN.2023.3289313)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_0347.pdf</t>
         </is>
       </c>
     </row>
@@ -9946,12 +9946,12 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1017.pdf</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -9976,7 +9976,7 @@
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/app132011278)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1017.pdf</t>
         </is>
       </c>
     </row>
@@ -10060,12 +10060,12 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1085.pdf</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/aerospace10030220)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1085.pdf</t>
         </is>
       </c>
     </row>
@@ -10117,12 +10117,12 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1118.pdf</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.1016/j.measurement.2022.112256)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1118.pdf</t>
         </is>
       </c>
     </row>
@@ -10174,12 +10174,12 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1135.pdf</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones7070451)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1135.pdf</t>
         </is>
       </c>
     </row>
@@ -10573,12 +10573,12 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1194.pdf</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -10603,7 +10603,7 @@
       </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones7100613)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1194.pdf</t>
         </is>
       </c>
     </row>
@@ -10630,12 +10630,12 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1196.pdf</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s23041934)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1196.pdf</t>
         </is>
       </c>
     </row>
@@ -10744,12 +10744,12 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1232.pdf</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones7080540)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1232.pdf</t>
         </is>
       </c>
     </row>
@@ -10801,12 +10801,12 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1250.pdf</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/aerospace10080708)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1250.pdf</t>
         </is>
       </c>
     </row>
@@ -11029,12 +11029,12 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1282.pdf</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -11059,7 +11059,7 @@
       </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/app13010414)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1282.pdf</t>
         </is>
       </c>
     </row>
@@ -11086,12 +11086,12 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1316.pdf</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/rs15215141)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1316.pdf</t>
         </is>
       </c>
     </row>
@@ -11200,12 +11200,12 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1402.pdf</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -11230,7 +11230,7 @@
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/drones7020073)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1402.pdf</t>
         </is>
       </c>
     </row>
@@ -11314,12 +11314,12 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1432.pdf</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="K147" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.2514/6.2023-2226)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1432.pdf</t>
         </is>
       </c>
     </row>
@@ -11485,12 +11485,12 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1455.pdf</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/app13148238)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1455.pdf</t>
         </is>
       </c>
     </row>
@@ -11827,12 +11827,12 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1660.pdf</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -11857,7 +11857,7 @@
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s23094366)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1660.pdf</t>
         </is>
       </c>
     </row>
@@ -12739,12 +12739,12 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1048.pdf</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -12769,7 +12769,7 @@
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s22093156)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1048.pdf</t>
         </is>
       </c>
     </row>
@@ -13081,12 +13081,12 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1289.pdf</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -13111,7 +13111,7 @@
       </c>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/aerospace9080456)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1289.pdf</t>
         </is>
       </c>
     </row>
@@ -13765,12 +13765,12 @@
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1587.pdf</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -13795,7 +13795,7 @@
       </c>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/s22249654)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1587.pdf</t>
         </is>
       </c>
     </row>
@@ -15418,12 +15418,12 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1059.pdf</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -15448,7 +15448,7 @@
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from Scopus (DOI: 10.3390/ijgi8040169)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_1059.pdf</t>
         </is>
       </c>
     </row>
@@ -18154,12 +18154,12 @@
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_0896.pdf</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -18184,7 +18184,7 @@
       </c>
       <c r="K267" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from IEEE_Xplore (DOI: 10.1109/ASCC.2017.8287144)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_0896.pdf</t>
         </is>
       </c>
     </row>
@@ -18838,12 +18838,12 @@
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>NOT_ON_DISK</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_0362.pdf</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
@@ -18868,7 +18868,7 @@
       </c>
       <c r="K279" s="2" t="inlineStr">
         <is>
-          <t>N - Pending download from IEEE_Xplore (DOI: 10.1109/PLANS.2016.7479719)</t>
+          <t>Y - PDF present in 05_papers_fulltext/REC_0362.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: integrate 6 newly staged PDFs (REC_1243, REC_0461, REC_1248, REC_1216, REC_1185, REC_1165); update PHASE1_MASTER.csv and PROJECT_MASTER_TRACKER.xlsx
</commit_message>
<xml_diff>
--- a/08_docs/PROJECT_MASTER_TRACKER.xlsx
+++ b/08_docs/PROJECT_MASTER_TRACKER.xlsx
@@ -7628,12 +7628,12 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -7643,12 +7643,12 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -7672,14 +7672,14 @@
         </is>
       </c>
       <c r="M70" s="3" t="inlineStr"/>
-      <c r="N70" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>REC_1165.pdf</t>
         </is>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1165.pdf</t>
         </is>
       </c>
       <c r="P70" s="3" t="inlineStr">
@@ -7944,12 +7944,12 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -7959,12 +7959,12 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -7988,14 +7988,14 @@
         </is>
       </c>
       <c r="M74" s="3" t="inlineStr"/>
-      <c r="N74" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>REC_1185.pdf</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1185.pdf</t>
         </is>
       </c>
       <c r="P74" s="3" t="inlineStr">
@@ -8102,12 +8102,12 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -8117,12 +8117,12 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -8146,14 +8146,14 @@
         </is>
       </c>
       <c r="M76" s="3" t="inlineStr"/>
-      <c r="N76" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>REC_1216.pdf</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1216.pdf</t>
         </is>
       </c>
       <c r="P76" s="3" t="inlineStr">
@@ -8339,12 +8339,12 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -8354,12 +8354,12 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
@@ -8383,14 +8383,14 @@
         </is>
       </c>
       <c r="M79" s="5" t="inlineStr"/>
-      <c r="N79" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t>REC_1243.pdf</t>
         </is>
       </c>
       <c r="O79" s="4" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1243.pdf</t>
         </is>
       </c>
       <c r="P79" s="5" t="inlineStr">
@@ -8418,12 +8418,12 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -8433,12 +8433,12 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -8462,14 +8462,14 @@
         </is>
       </c>
       <c r="M80" s="3" t="inlineStr"/>
-      <c r="N80" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>REC_1248.pdf</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1248.pdf</t>
         </is>
       </c>
       <c r="P80" s="3" t="inlineStr">
@@ -25719,12 +25719,12 @@
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E299" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F299" s="5" t="inlineStr">
@@ -25734,12 +25734,12 @@
       </c>
       <c r="G299" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I299" s="4" t="inlineStr">
@@ -25763,14 +25763,14 @@
         </is>
       </c>
       <c r="M299" s="5" t="inlineStr"/>
-      <c r="N299" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N299" s="4" t="inlineStr">
+        <is>
+          <t>REC_0461.pdf</t>
         </is>
       </c>
       <c r="O299" s="4" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_0461.pdf</t>
         </is>
       </c>
       <c r="P299" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs: integrate 5 newly downloaded PDFs (REC_1187, REC_1322, REC_1608, REC_1336, REC_1541); update tracker to 252/300 (84.0%)
</commit_message>
<xml_diff>
--- a/08_docs/PROJECT_MASTER_TRACKER.xlsx
+++ b/08_docs/PROJECT_MASTER_TRACKER.xlsx
@@ -20189,12 +20189,12 @@
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E229" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F229" s="5" t="inlineStr">
@@ -20204,12 +20204,12 @@
       </c>
       <c r="G229" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H229" s="4" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I229" s="5" t="inlineStr">
@@ -20233,14 +20233,14 @@
         </is>
       </c>
       <c r="M229" s="5" t="inlineStr"/>
-      <c r="N229" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N229" s="4" t="inlineStr">
+        <is>
+          <t>REC_1541.pdf</t>
         </is>
       </c>
       <c r="O229" s="4" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1541.pdf</t>
         </is>
       </c>
       <c r="P229" s="5" t="inlineStr">
@@ -24613,12 +24613,12 @@
       </c>
       <c r="D285" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E285" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
@@ -24628,12 +24628,12 @@
       </c>
       <c r="G285" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I285" s="5" t="inlineStr">
@@ -24657,14 +24657,14 @@
         </is>
       </c>
       <c r="M285" s="5" t="inlineStr"/>
-      <c r="N285" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N285" s="4" t="inlineStr">
+        <is>
+          <t>REC_1187.pdf</t>
         </is>
       </c>
       <c r="O285" s="4" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1187.pdf</t>
         </is>
       </c>
       <c r="P285" s="5" t="inlineStr">
@@ -24692,12 +24692,12 @@
       </c>
       <c r="D286" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E286" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F286" s="3" t="inlineStr">
@@ -24707,12 +24707,12 @@
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I286" s="3" t="inlineStr">
@@ -24736,14 +24736,14 @@
         </is>
       </c>
       <c r="M286" s="3" t="inlineStr"/>
-      <c r="N286" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N286" s="2" t="inlineStr">
+        <is>
+          <t>REC_1322.pdf</t>
         </is>
       </c>
       <c r="O286" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1322.pdf</t>
         </is>
       </c>
       <c r="P286" s="3" t="inlineStr">
@@ -24771,12 +24771,12 @@
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E287" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
@@ -24786,12 +24786,12 @@
       </c>
       <c r="G287" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I287" s="5" t="inlineStr">
@@ -24815,14 +24815,14 @@
         </is>
       </c>
       <c r="M287" s="5" t="inlineStr"/>
-      <c r="N287" s="5" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N287" s="4" t="inlineStr">
+        <is>
+          <t>REC_1336.pdf</t>
         </is>
       </c>
       <c r="O287" s="4" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1336.pdf</t>
         </is>
       </c>
       <c r="P287" s="5" t="inlineStr">
@@ -25324,12 +25324,12 @@
       </c>
       <c r="D294" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E294" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F294" s="3" t="inlineStr">
@@ -25339,12 +25339,12 @@
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>Truly_pending</t>
+          <t>PDF_present_master_missing</t>
         </is>
       </c>
       <c r="I294" s="3" t="inlineStr">
@@ -25368,14 +25368,14 @@
         </is>
       </c>
       <c r="M294" s="3" t="inlineStr"/>
-      <c r="N294" s="3" t="inlineStr">
-        <is>
-          <t>NONE</t>
+      <c r="N294" s="2" t="inlineStr">
+        <is>
+          <t>REC_1608.pdf</t>
         </is>
       </c>
       <c r="O294" s="2" t="inlineStr">
         <is>
-          <t>N/A (Missing)</t>
+          <t>E:\GPS_Denied_SLR\05_papers_fulltext\REC_1608.pdf</t>
         </is>
       </c>
       <c r="P294" s="3" t="inlineStr">

</xml_diff>